<commit_message>
Şablonlarda yalnızca ilgili toleransı göster
Birim fiyatlı işte pursantaj olmadığı için BFTC şablonundan pursantaj
toleransı, anahtar teslim şablonundan kullanılmayan metraj toleransı
kaldırıldı.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HeSgjaumyie6wfCEgGCs7w
</commit_message>
<xml_diff>
--- a/ihale-analiz/templates/excel/anahtar-teslim.xlsx
+++ b/ihale-analiz/templates/excel/anahtar-teslim.xlsx
@@ -20,8 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_harita" sheetId="11" state="hidden" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="MetrajTol">'Özet'!$B$17</definedName>
-    <definedName name="PursantajTol">'Özet'!$B$18</definedName>
+    <definedName name="PursantajTol">'Özet'!$B$17</definedName>
     <definedName name="YaklasikMaliyet">'Özet'!$B$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mahal Listesi'!$A$4:$M$504</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Mahal Listesi'!$4:$4</definedName>
@@ -600,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -836,30 +835,20 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Metraj Toleransı</t>
+          <t>Pursantaj Toleransı (puan)</t>
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Pursantaj Toleransı (puan)</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
           <t>Analiz Tarihi</t>
         </is>
       </c>
-      <c r="B19" s="13" t="n"/>
+      <c r="B18" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>